<commit_message>
feat: v0.3.3 UI polish — run lifecycle, update checker, language logos, status bar
Undo-revert for saved snapshots, run lifecycle (Saving→Compiling→Running)
in console and status bar, close-dirty-tab dialog, book chapter "Read Online"
links, VS Code-style status bar, toolbar reorganization, dynamic window title,
update checker via GitHub Releases API, official language SVG logos replacing
text badges across Sidebar/ProjectSwitcher/ToolchainWizard/toolbar, cargo logo
for Rust toolchain, dark-mode invert for Rust logo, book auto-select on
language enable, reactive book labels, min window width 900px. Docs updated.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/testing/TESTING-LOG-v0.3.3-Rust-Edition-2026-04-05-jagmeet.xlsx
+++ b/testing/TESTING-LOG-v0.3.3-Rust-Edition-2026-04-05-jagmeet.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -46,6 +46,10 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -87,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -95,6 +99,7 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -475,7 +480,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
     </row>
@@ -533,7 +538,6 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -541,7 +545,6 @@
           <t>macOS version</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -549,7 +552,6 @@
           <t>Xcode CLT version</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
@@ -557,7 +559,6 @@
           <t>Tester</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
@@ -582,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D227"/>
+  <dimension ref="A1:D284"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -605,6 +606,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -3430,6 +3432,571 @@
       </c>
       <c r="C227" s="6" t="n"/>
       <c r="D227" s="6" t="n"/>
+    </row>
+    <row r="229">
+      <c r="A229" s="7" t="inlineStr">
+        <is>
+          <t>SAVED SNAPSHOT SYSTEM &amp; REVERT</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B230" s="1" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="C230" s="1" t="inlineStr">
+        <is>
+          <t>Pass?</t>
+        </is>
+      </c>
+      <c r="D230" s="1" t="inlineStr">
+        <is>
+          <t>Notes / Screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="n">
+        <v>192</v>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>Edit playground → dirty dot appears on tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="n">
+        <v>193</v>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>Revert (toolbar button) → code restored to saved version</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="n">
+        <v>194</v>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Revert → dirty dot removed from tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="n">
+        <v>195</v>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Revert → button changes to 'Undo Revert'</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="n">
+        <v>196</v>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Undo Revert → dirty code restored, dirty dot returns</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="n">
+        <v>197</v>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Undo Revert → button changes back to 'Revert'</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="n">
+        <v>198</v>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>Start typing after revert → Undo Revert disappears</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="n">
+        <v>199</v>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>Close dirty tab → Save / Don't Save / Cancel dialog</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="n">
+        <v>200</v>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Close dirty tab → Save → file saved, tab closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="n">
+        <v>201</v>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>Close dirty tab → Don't Save → changes discarded, tab closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="n">
+        <v>202</v>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Close dirty tab → Cancel → tab stays open, changes intact</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="n">
+        <v>203</v>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>Edit → close without save → reopen → clean saved code (snapshot system)</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="n">
+        <v>204</v>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>Run with unsaved changes → auto-saves before compile</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="7" t="inlineStr">
+        <is>
+          <t>RUN LIFECYCLE STATUS</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B246" s="1" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="C246" s="1" t="inlineStr">
+        <is>
+          <t>Pass?</t>
+        </is>
+      </c>
+      <c r="D246" s="1" t="inlineStr">
+        <is>
+          <t>Notes / Screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="n">
+        <v>205</v>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>Run → console shows 'Saving…' info line</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="n">
+        <v>206</v>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>Run → console shows 'Compiling…' info line after save</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="n">
+        <v>207</v>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>Run → console shows 'Running…' info line when program starts</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="n">
+        <v>208</v>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>All three info lines have timestamps</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="n">
+        <v>209</v>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>Status bar below editor shows 'Saving…' → 'Compiling…' → 'Running��'</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="n">
+        <v>210</v>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>Build failure → status bar shows 'Build failed'</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="n">
+        <v>211</v>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>Status bar hidden when idle (no run in progress)</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="7" t="inlineStr">
+        <is>
+          <t>READ ONLINE — BOOK CHAPTER LINK</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B256" s="1" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="C256" s="1" t="inlineStr">
+        <is>
+          <t>Pass?</t>
+        </is>
+      </c>
+      <c r="D256" s="1" t="inlineStr">
+        <is>
+          <t>Notes / Screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="n">
+        <v>212</v>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Select book chapter → 'Read Online' link in status bar</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="n">
+        <v>213</v>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Click 'Read Online' → opens correct chapter in browser</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="n">
+        <v>214</v>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Ch 1 → https://doc.rust-lang.org/book/ch01-00-getting-started.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="n">
+        <v>215</v>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Switch to user project → 'Read Online' disappears</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="n">
+        <v>216</v>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>Switch between chapters → link updates correctly</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="7" t="inlineStr">
+        <is>
+          <t>TOOLBAR LAYOUT &amp; WINDOW TITLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B264" s="1" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="C264" s="1" t="inlineStr">
+        <is>
+          <t>Pass?</t>
+        </is>
+      </c>
+      <c r="D264" s="1" t="inlineStr">
+        <is>
+          <t>Notes / Screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="n">
+        <v>217</v>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>Toolchain pill is left-aligned (next to project switcher)</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="n">
+        <v>218</v>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>Settings gear icon in toolbar-right (no border/background)</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="n">
+        <v>219</v>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>Settings gear opens Settings modal (⌘,)</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="n">
+        <v>220</v>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>Window title: 'Rustic Rust' on launch</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="n">
+        <v>221</v>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>Window title: 'Rustic Rust — project_name' when project selected</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="n">
+        <v>222</v>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>Window title: 'Rustic Rust — project — playground' when tab open</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="n">
+        <v>223</v>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>Window title updates when switching projects/tabs</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="n">
+        <v>224</v>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>Minimum window width is 900px (can't resize smaller)</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="n">
+        <v>225</v>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>Toolbar controls don't overlap at minimum width</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="7" t="inlineStr">
+        <is>
+          <t>BOOK AUTO-SELECT &amp; REACTIVE LABELS</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B276" s="1" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="C276" s="1" t="inlineStr">
+        <is>
+          <t>Pass?</t>
+        </is>
+      </c>
+      <c r="D276" s="1" t="inlineStr">
+        <is>
+          <t>Notes / Screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="n">
+        <v>226</v>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>Settings → Languages: enable language with book → book auto-checked</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="n">
+        <v>227</v>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>Settings → Languages: disable language → book hidden from Books tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="n">
+        <v>228</v>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>Settings → Languages: re-enable language → book still checked</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="n">
+        <v>229</v>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>Settings → Books tab: manually uncheck book → stays unchecked</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="n">
+        <v>230</v>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>Settings → Apply with language disabled → its book removed</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="n">
+        <v>231</v>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>Book/Books tab label: 1 book language = 'Book', 2+ = 'Books'</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="n">
+        <v>232</v>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>Label updates live as languages toggled (no need to close/reopen)</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="n">
+        <v>233</v>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>0 book languages → Books tab disappears, redirects to Appearance</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>